<commit_message>
Add Improve Traffic regression suites, portal automation plan, and Allure reports.
Expand US2 coverage with Brand/Sales Customer Journey Analysis and Core Web Vitals suites, shared CJA POM support, Excel workbooks, leadership plan generator, and latest Allure HTML reports.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Marketing_Overview_Regression.xlsx
+++ b/docs/Marketing_Overview_Regression.xlsx
@@ -477,14 +477,23 @@
     <t>No layout mutation on shared dashboard</t>
   </si>
   <si>
-    <t>Reset Widgets control present but not clicked</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Locate #reset-all-inactive-widgets
-2. Do not click on shared dashboard</t>
-  </si>
-  <si>
-    <t>Control presence documented; no reset executed</t>
+    <t>Hide Widget, Reset behavior, and hidden-widget recovery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Hide the Campaigns widget and confirm Hide Widget
+2. Verify Campaigns is removed from the active grid
+3. Click Reset Widgets and confirm Reset All Widgets
+4. Record whether Reset restores the hidden widget
+5. If Reset only restores positions, expand hidden widgets and drag Campaigns back
+6. Repeat for Campaigns Over Time
+7. Verify both widgets and their data are restored</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each selected widget is hidden after confirmation
+Reset Widgets behavior is captured independently for each widget
+A widget not unhidden by Reset is restored from the hidden-widget panel
+Campaign cards and Campaigns Over Time bar/line graphs are healthy after recovery
+The shared dashboard is not left with hidden widgets</t>
   </si>
   <si>
     <t>REG-MO-021</t>
@@ -561,16 +570,25 @@
     <t>REG-MO-027</t>
   </si>
   <si>
-    <t>Select each campaign metric and assert graph signature updates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Select each metric
-2. Compare scoped graph signatures
-3. Restore original metric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Active metric state updates
-Graph signature captured before/after</t>
+    <t>Every Campaigns Over Time tab has graph data and detailed tooltips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Capture the original active metric and bar/line graph signatures
+2. Select Revenue, Orders, Avg Order Value, Conversion Rate, Bounce Rate, Exit Rate, and Sessions in turn
+3. Verify the selected tab becomes active
+4. Verify both scoped bar and line graphs contain non-null data points
+5. Hover representative points on both graphs
+6. Validate tooltip details and units: currency for Revenue/AOV, percentages for rates, counts for Orders/Sessions
+7. Record any stale metric/unit tooltip behavior without skipping remaining tabs
+8. Restore the original metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All seven metric tabs exist and are selectable
+Both graphs contain live data for every data-bearing metric
+Bar and line tooltips contain campaign/time/value details
+Tooltip units correspond to the active metric
+All tabs are exercised even if one tab produces a soft live-UI finding
+Original metric is restored</t>
   </si>
   <si>
     <t>REG-MO-028</t>
@@ -625,14 +643,21 @@
     <t>REG-MO-032</t>
   </si>
   <si>
-    <t>Campaign graph context/export menu opens and dismisses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open context menu on bar graph
-2. Dismiss with Escape</t>
-  </si>
-  <si>
-    <t>Menu dismisses; no blocking overlay</t>
+    <t>Campaigns Over Time hamburger options work and restore chart state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the hamburger menu scoped to the Campaigns Over Time bar graph
+2. Verify View in Full Screen, Toggle Data Labels, and Download PNG Image options
+3. Invoke Toggle Data Labels
+4. Verify the chart remains rendered and interactive
+5. Invoke Toggle Data Labels again to restore the original state
+6. Dismiss menus and verify no overlay blocks dashboard controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected chart menu options are available
+Toggle Data Labels action is accepted and can be reversed
+Chart remains healthy after menu actions
+Menu closes without leaving a blocking overlay</t>
   </si>
   <si>
     <t>REG-MO-033</t>
@@ -655,26 +680,39 @@
     <t>Source table sort / search / clear when rows exist</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Sort Revenue
-2. Search runtime-derived source
-3. No-match then clear</t>
-  </si>
-  <si>
-    <t>Row order/search behavior validated when data present</t>
+    <t xml:space="preserve">1. If the Source table has rows, capture the visible row signature
+2. Sort Revenue; reverse direction if the first click preserves the existing order
+3. Verify visible row order changes
+4. Search using a runtime-derived source value
+5. Apply a guaranteed no-match term
+6. Clear search and restore the table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue sorting changes actual row order when multiple rows exist
+Runtime-derived search limits rows correctly
+No-match search shows a controlled empty result
+Clear restores rows
+Scenario is annotated when the Source table is absent/empty</t>
   </si>
   <si>
     <t>REG-MO-035</t>
   </si>
   <si>
-    <t>Source table page-size and export options when present</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Change page size
-2. Open Export menu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Page-size applies when present
-Export includes CSV/TSV/JSON/Array when present</t>
+    <t>Source table page-size, Next/Previous pagination, and export options</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. If the Source table is present, change page size to a configured value
+2. If Next is enabled, capture the current row/pager signature and click Next
+3. Verify the visible page changes
+4. Click Previous and verify the original page is restored
+5. Open Export and verify CSV, TSV, JSON, and Array options when configured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page-size selection applies
+Next/Previous changes and restores visible rows when multiple pages exist
+Single-page state is handled without failure
+Configured export options are present
+Scenario is annotated when the Source table is unavailable</t>
   </si>
   <si>
     <t>REG-MO-036</t>
@@ -694,15 +732,22 @@
     <t>REG-MO-037</t>
   </si>
   <si>
-    <t>Medium table sort / search / page-size / export</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Sort Orders
-2. Change page size
-3. Open Export</t>
-  </si>
-  <si>
-    <t>Interactions succeed; export options when present</t>
+    <t>Medium table sorting, search, page-size, pagination, and export</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. If the Medium table has rows, capture its visible row signature
+2. Sort Orders ascending/descending and verify row-order change
+3. Exercise runtime-derived search and clear when available
+4. Change page size
+5. Exercise enabled Next/Previous and verify page restoration
+6. Open Export and inspect configured formats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorting changes actual row order when multiple rows exist
+Search and clear preserve table usability
+Page-size and enabled pagination work
+Export options are available when configured
+Scenario is annotated when the Medium table is absent/empty</t>
   </si>
   <si>
     <t>REG-MO-038</t>
@@ -746,14 +791,23 @@
 Legend toggle restores</t>
   </si>
   <si>
-    <t>Device graph context menus dismiss without overlay block</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Open context menus
-2. Escape/dismiss</t>
-  </si>
-  <si>
-    <t>No blocking overlay; refresh control usable</t>
+    <t>Hamburger options work independently on different device widgets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the hamburger menu on Revenue by Device
+2. Verify chart/export options and toggle data labels on/off
+3. Open the hamburger menu on Conversion Rate by Device
+4. Invoke View in Full Screen and exit with Escape
+5. Open the hamburger menu on Sessions by Device
+6. Verify the menu is scoped to that chart and dismiss it
+7. Confirm dashboard controls remain usable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each device widget exposes its own hamburger menu
+Expected image export and chart interaction options are available
+Safe actions execute without corrupting other widgets
+Data-label/fullscreen state is restored
+No menu overlay blocks the dashboard</t>
   </si>
   <si>
     <t>REG-MO-042</t>
@@ -878,7 +932,7 @@
     <t>Profile / Site: US — GDC Test Site 2</t>
   </si>
   <si>
-    <t>Type: Regression (read-only). Do NOT Save Filter, create markers, Reset Widgets, edit/delete dashboards, or switch users.</t>
+    <t>Type: Regression. Do NOT Save Filter, create markers, edit/delete dashboards, or switch users. The controlled Hide Widget / Reset Widgets scenario must restore every hidden widget before continuing.</t>
   </si>
   <si>
     <t>Do not hard-code dashboard name, lookback, campaign names, or metric totals.</t>
@@ -896,10 +950,10 @@
     <t>Execution status: Pass</t>
   </si>
   <si>
-    <t>Execution note: Isolated run 2026-07-30: 51 passed (50 REG-MO + auth). Soft annotations: Source/Medium tables not present on live _BTT Marketing Overview layout; Event Markers may be annotated when menu mis-resolves; Tablet series data-dependent; dashboard name and lookback captured dynamically (Last 6 hours at run time).</t>
-  </si>
-  <si>
-    <t>Ambiguities: dashboard "_BTT Marketing Overview" may be site-specific; Source table may be empty; Tablet series may be empty; Viewing/Editing read-only only.</t>
+    <t>Execution note: Latest automated run: 51 passed (50 REG-MO cases plus authentication). Source/Medium tables were unavailable. Soft findings: Orders tooltip retained currency, AOV occasionally remained on Revenue, and Sessions tooltip showed percentage formatting. See allure_reports/marketing-overview-report/index.html.</t>
+  </si>
+  <si>
+    <t>Live findings: Reset Widgets may restore positions without consistently unhiding every widget; use the hidden-widget panel for recovery. Source/Medium tables may be absent. Orders/Sessions tooltip units and AOV active-state behavior are recorded as soft findings when stale.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Add Native App Detailed Metrics dashboard regression and related tooling.
Include the Android-home multi-widget suite (soft iOS dual), live probes and AI prompts for Native App Detailed Metrics and Performance Detail, shared manual Excel format helpers, and stability heals for Session Lookup, Performance Overview, Performance Budget, VitalPulse, and Bottom Sales Funnel.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Marketing_Overview_Regression.xlsx
+++ b/docs/Marketing_Overview_Regression.xlsx
@@ -13,12 +13,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="266">
-  <si>
-    <t>Marketing Overview Regression — GDC Test Site 2 (US)</t>
-  </si>
-  <si>
-    <t>Help / DOC: The Marketing Overview Page – Blue Triangle Help Center (attached PDF / Help Center)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="264">
+  <si>
+    <t>Profile: US / GDC Test Site 2 | Type: Regression (read-only) | Total TCs: 50 | Marketing Overview</t>
+  </si>
+  <si>
+    <t>tests/regression_tests/US2/business-insights/improve-traffic/marketing-overview/marketing.overview.regression.spec.ts</t>
   </si>
   <si>
     <t>Module</t>
@@ -231,9 +231,9 @@
 4. Observe breadcrumb and URL</t>
   </si>
   <si>
-    <t xml:space="preserve">Breadcrumb: Business Insights / Improve Traffic / Marketing Overview
-URL contains overview-dashboard/marketing
-No login redirect</t>
+    <t xml:space="preserve">1. Breadcrumb: Business Insights / Improve Traffic / Marketing Overview
+2. URL contains overview-dashboard/marketing
+3. No login redirect</t>
   </si>
   <si>
     <t>Pass</t>
@@ -247,9 +247,9 @@
 3. Do not assume a fixed default period (e.g. Last 6 Hours or 30 days)</t>
   </si>
   <si>
-    <t xml:space="preserve">Site is GDC Test Site 2
-Dashboard and lookback labels are non-empty live values
-Sitewide Totals and widgets render</t>
+    <t xml:space="preserve">1. Site is GDC Test Site 2
+2. Dashboard and lookback labels are non-empty live values
+3. Sitewide Totals and widgets render</t>
   </si>
   <si>
     <t>Sitewide Totals and at least one marketing widget render</t>
@@ -258,8 +258,8 @@
     <t>1. After page ready, observe Sitewide Totals and Campaigns/charts</t>
   </si>
   <si>
-    <t xml:space="preserve">Sitewide Totals visible
-At least one campaign card or Highcharts container present</t>
+    <t xml:space="preserve">1. Sitewide Totals visible
+2. At least one campaign card or Highcharts container present</t>
   </si>
   <si>
     <t>Primary widgets finish loading within bounded UI deadline</t>
@@ -268,7 +268,7 @@
     <t>1. Measure warm-session navigation until widgets ready</t>
   </si>
   <si>
-    <t>Ready within 120 seconds UI observation (not a formal backend SLA)</t>
+    <t>1. Ready within 120 seconds UI observation (not a formal backend SLA)</t>
   </si>
   <si>
     <t>REG-MO-005</t>
@@ -280,7 +280,7 @@
     <t>1. Observe document title</t>
   </si>
   <si>
-    <t>Title contains Marketing</t>
+    <t>1. Title contains Marketing</t>
   </si>
   <si>
     <t>REG-MO-006</t>
@@ -293,7 +293,7 @@
 2. Verify markers / reset / view-or-edit when configured</t>
   </si>
   <si>
-    <t>Configured controls visible or attached with accessible names/tooltips</t>
+    <t>1. Configured controls visible or attached with accessible names/tooltips</t>
   </si>
   <si>
     <t>REG-MO-007</t>
@@ -305,8 +305,8 @@
     <t>1. Enumerate #switch-dashboard options</t>
   </si>
   <si>
-    <t xml:space="preserve">No blank or duplicate option labels
-Selected dashboard non-empty</t>
+    <t xml:space="preserve">1. No blank or duplicate option labels
+2. Selected dashboard non-empty</t>
   </si>
   <si>
     <t>Manual refresh reloads widgets without duplication</t>
@@ -317,9 +317,9 @@
 3. Wait for reload</t>
   </si>
   <si>
-    <t xml:space="preserve">Widgets reload
-No duplicate graph host IDs
-Controls usable again</t>
+    <t xml:space="preserve">1. Widgets reload
+2. No duplicate graph host IDs
+3. Controls usable again</t>
   </si>
   <si>
     <t>REG-MO-009</t>
@@ -332,8 +332,8 @@
 2. Enumerate all presets</t>
   </si>
   <si>
-    <t xml:space="preserve">Presets unique and non-blank
-Record live list</t>
+    <t xml:space="preserve">1. Presets unique and non-blank
+2. Record live list</t>
   </si>
   <si>
     <t>REG-MO-010</t>
@@ -347,9 +347,9 @@
 3. Compare totals</t>
   </si>
   <si>
-    <t xml:space="preserve">Selected label changes
-Totals/widget state refreshes
-Annotate if preset missing</t>
+    <t xml:space="preserve">1. Selected label changes
+2. Totals/widget state refreshes
+3. Annotate if preset missing</t>
   </si>
   <si>
     <t>REG-MO-011</t>
@@ -362,7 +362,7 @@
 2. Compare campaign card signature</t>
   </si>
   <si>
-    <t>Widgets reload for selected period</t>
+    <t>1. Widgets reload for selected period</t>
   </si>
   <si>
     <t>REG-MO-012</t>
@@ -376,7 +376,8 @@
 3. Compare graph signature</t>
   </si>
   <si>
-    <t>Bar/line graphs refresh; do not only count containers</t>
+    <t xml:space="preserve">1. Bar/line graphs refresh
+2. do not only count containers</t>
   </si>
   <si>
     <t>REG-MO-013</t>
@@ -389,8 +390,8 @@
 2. Restore originally captured lookback</t>
   </si>
   <si>
-    <t xml:space="preserve">Period applies when available
-Original lookback restored</t>
+    <t xml:space="preserve">1. Period applies when available
+2. Original lookback restored</t>
   </si>
   <si>
     <t>REG-MO-014</t>
@@ -403,8 +404,8 @@
 2. Cancel without applying</t>
   </si>
   <si>
-    <t xml:space="preserve">Lookback remains a valid prior/selected value
-No stuck overlay</t>
+    <t xml:space="preserve">1. Lookback remains a valid prior/selected value
+2. No stuck overlay</t>
   </si>
   <si>
     <t>REG-MO-015</t>
@@ -419,9 +420,9 @@
 4. Do not wait full interval</t>
   </si>
   <si>
-    <t xml:space="preserve">Options unique
-Label updates
-Original restored</t>
+    <t xml:space="preserve">1. Options unique
+2. Label updates
+3. Original restored</t>
   </si>
   <si>
     <t>REG-MO-016</t>
@@ -435,7 +436,7 @@
 3. Confirm lookback unchanged</t>
   </si>
   <si>
-    <t>Lookback unchanged</t>
+    <t>1. Lookback unchanged</t>
   </si>
   <si>
     <t>Event Markers options sample and restore (no create/edit/delete)</t>
@@ -446,9 +447,9 @@
 3. Do not Create A New Marker</t>
   </si>
   <si>
-    <t xml:space="preserve">Options valid
-Charts update marker visibility when applicable
-Original restored</t>
+    <t xml:space="preserve">1. Options valid
+2. Charts update marker visibility when applicable
+3. Original restored</t>
   </si>
   <si>
     <t>REG-MO-018</t>
@@ -461,7 +462,7 @@
 2. Inspect drag/edit handles</t>
   </si>
   <si>
-    <t>Drag/edit handles not active in Viewing</t>
+    <t>1. Drag/edit handles not active in Viewing</t>
   </si>
   <si>
     <t>REG-MO-019</t>
@@ -474,7 +475,7 @@
 2. Return to Viewing without moving widgets</t>
   </si>
   <si>
-    <t>No layout mutation on shared dashboard</t>
+    <t>1. No layout mutation on shared dashboard</t>
   </si>
   <si>
     <t>Hide Widget, Reset behavior, and hidden-widget recovery</t>
@@ -489,11 +490,11 @@
 7. Verify both widgets and their data are restored</t>
   </si>
   <si>
-    <t xml:space="preserve">Each selected widget is hidden after confirmation
-Reset Widgets behavior is captured independently for each widget
-A widget not unhidden by Reset is restored from the hidden-widget panel
-Campaign cards and Campaigns Over Time bar/line graphs are healthy after recovery
-The shared dashboard is not left with hidden widgets</t>
+    <t xml:space="preserve">1. Each selected widget is hidden after confirmation
+2. Reset Widgets behavior is captured independently for each widget
+3. A widget not unhidden by Reset is restored from the hidden-widget panel
+4. Campaign cards and Campaigns Over Time bar/line graphs are healthy after recovery
+5. The shared dashboard is not left with hidden widgets</t>
   </si>
   <si>
     <t>REG-MO-021</t>
@@ -505,7 +506,7 @@
     <t>1. Verify title and cards #bounce-rate-card … #conversion-rate-card</t>
   </si>
   <si>
-    <t>All ten cards attached with non-empty value or controlled no-data</t>
+    <t>1. All ten cards attached with non-empty value or controlled no-data</t>
   </si>
   <si>
     <t>REG-MO-022</t>
@@ -517,7 +518,7 @@
     <t>1. Sample Bounce Rate, Revenue, Sessions, Onload formats</t>
   </si>
   <si>
-    <t>Formats match type (%, currency/count, duration) without exact values</t>
+    <t>1. Formats match type (%, currency/count, duration) without exact values</t>
   </si>
   <si>
     <t>REG-MO-023</t>
@@ -529,7 +530,7 @@
     <t>1. Hover info icons on metric cards</t>
   </si>
   <si>
-    <t>Meaningful tooltip/title text when icons present</t>
+    <t>1. Meaningful tooltip/title text when icons present</t>
   </si>
   <si>
     <t>Campaigns widget shows at least one data-bearing card</t>
@@ -539,7 +540,7 @@
 2. Validate non-empty labels/metrics</t>
   </si>
   <si>
-    <t>At least one card OR annotate controlled no-data</t>
+    <t>1. At least one card OR annotate controlled no-data</t>
   </si>
   <si>
     <t>Campaign action menu labels and safe Back navigation</t>
@@ -551,8 +552,8 @@
 4. Close extra tabs</t>
   </si>
   <si>
-    <t xml:space="preserve">Menu labels present
-Marketing Overview restores after Back</t>
+    <t xml:space="preserve">1. Menu labels present
+2. Marketing Overview restores after Back</t>
   </si>
   <si>
     <t>REG-MO-026</t>
@@ -564,7 +565,7 @@
     <t>1. Verify #revenue-campaigns … #sessions-campaigns</t>
   </si>
   <si>
-    <t>All configured metric buttons visible</t>
+    <t>1. All configured metric buttons visible</t>
   </si>
   <si>
     <t>REG-MO-027</t>
@@ -583,12 +584,12 @@
 8. Restore the original metric</t>
   </si>
   <si>
-    <t xml:space="preserve">All seven metric tabs exist and are selectable
-Both graphs contain live data for every data-bearing metric
-Bar and line tooltips contain campaign/time/value details
-Tooltip units correspond to the active metric
-All tabs are exercised even if one tab produces a soft live-UI finding
-Original metric is restored</t>
+    <t xml:space="preserve">1. All seven metric tabs exist and are selectable
+2. Both graphs contain live data for every data-bearing metric
+3. Bar and line tooltips contain campaign/time/value details
+4. Tooltip units correspond to the active metric
+5. All tabs are exercised even if one tab produces a soft live-UI finding
+6. Original metric is restored</t>
   </si>
   <si>
     <t>REG-MO-028</t>
@@ -600,7 +601,7 @@
     <t>1. Rapidly click Orders → Sessions → Revenue</t>
   </si>
   <si>
-    <t>Final active metric is Revenue</t>
+    <t>1. Final active metric is Revenue</t>
   </si>
   <si>
     <t>REG-MO-029</t>
@@ -612,7 +613,7 @@
     <t>1. Verify #top-campaigns-by-campaign-bar and -line</t>
   </si>
   <si>
-    <t>Both graphs render for data-bearing metric</t>
+    <t>1. Both graphs render for data-bearing metric</t>
   </si>
   <si>
     <t>REG-MO-030</t>
@@ -625,7 +626,7 @@
 2. Read tooltip fields</t>
   </si>
   <si>
-    <t>Tooltip content asserted when available</t>
+    <t>1. Tooltip content asserted when available</t>
   </si>
   <si>
     <t>REG-MO-031</t>
@@ -637,7 +638,7 @@
     <t>1. Toggle first legend item twice</t>
   </si>
   <si>
-    <t>Series visibility changes and restores</t>
+    <t>1. Series visibility changes and restores</t>
   </si>
   <si>
     <t>REG-MO-032</t>
@@ -654,10 +655,10 @@
 6. Dismiss menus and verify no overlay blocks dashboard controls</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected chart menu options are available
-Toggle Data Labels action is accepted and can be reversed
-Chart remains healthy after menu actions
-Menu closes without leaving a blocking overlay</t>
+    <t xml:space="preserve">1. Expected chart menu options are available
+2. Toggle Data Labels action is accepted and can be reversed
+3. Chart remains healthy after menu actions
+4. Menu closes without leaving a blocking overlay</t>
   </si>
   <si>
     <t>REG-MO-033</t>
@@ -670,8 +671,8 @@
 2. Verify columns</t>
   </si>
   <si>
-    <t xml:space="preserve">Headers: Source, Revenue ($), Orders, Avg Order Value ($), Visitors, Page Views, Conversion Rate (%)
-Rows OR controlled empty annotated</t>
+    <t xml:space="preserve">1. Headers: Source, Revenue ($), Orders, Avg Order Value ($), Visitors, Page Views, Conversion Rate (%)
+2. Rows OR controlled empty annotated</t>
   </si>
   <si>
     <t>REG-MO-034</t>
@@ -688,11 +689,11 @@
 6. Clear search and restore the table</t>
   </si>
   <si>
-    <t xml:space="preserve">Revenue sorting changes actual row order when multiple rows exist
-Runtime-derived search limits rows correctly
-No-match search shows a controlled empty result
-Clear restores rows
-Scenario is annotated when the Source table is absent/empty</t>
+    <t xml:space="preserve">1. Revenue sorting changes actual row order when multiple rows exist
+2. Runtime-derived search limits rows correctly
+3. No-match search shows a controlled empty result
+4. Clear restores rows
+5. Scenario is annotated when the Source table is absent/empty</t>
   </si>
   <si>
     <t>REG-MO-035</t>
@@ -708,11 +709,11 @@
 5. Open Export and verify CSV, TSV, JSON, and Array options when configured</t>
   </si>
   <si>
-    <t xml:space="preserve">Page-size selection applies
-Next/Previous changes and restores visible rows when multiple pages exist
-Single-page state is handled without failure
-Configured export options are present
-Scenario is annotated when the Source table is unavailable</t>
+    <t xml:space="preserve">1. Page-size selection applies
+2. Next/Previous changes and restores visible rows when multiple pages exist
+3. Single-page state is handled without failure
+4. Configured export options are present
+5. Scenario is annotated when the Source table is unavailable</t>
   </si>
   <si>
     <t>REG-MO-036</t>
@@ -725,8 +726,8 @@
 2. Verify columns and sample rows</t>
   </si>
   <si>
-    <t xml:space="preserve">Stable headers present
-Formats validated without exact values</t>
+    <t xml:space="preserve">1. Stable headers present
+2. Formats validated without exact values</t>
   </si>
   <si>
     <t>REG-MO-037</t>
@@ -743,11 +744,11 @@
 6. Open Export and inspect configured formats</t>
   </si>
   <si>
-    <t xml:space="preserve">Sorting changes actual row order when multiple rows exist
-Search and clear preserve table usability
-Page-size and enabled pagination work
-Export options are available when configured
-Scenario is annotated when the Medium table is absent/empty</t>
+    <t xml:space="preserve">1. Sorting changes actual row order when multiple rows exist
+2. Search and clear preserve table usability
+3. Page-size and enabled pagination work
+4. Export options are available when configured
+5. Scenario is annotated when the Medium table is absent/empty</t>
   </si>
   <si>
     <t>REG-MO-038</t>
@@ -760,8 +761,8 @@
 2. Hover sample point</t>
   </si>
   <si>
-    <t xml:space="preserve">Graphs render
-Desktop/Mobile/Tablet series data-dependent</t>
+    <t xml:space="preserve">1. Graphs render
+2. Desktop/Mobile/Tablet series data-dependent</t>
   </si>
   <si>
     <t>REG-MO-039</t>
@@ -774,7 +775,7 @@
 2. Hover tooltip</t>
   </si>
   <si>
-    <t>Percentage presentation without exact backend values</t>
+    <t>1. Percentage presentation without exact backend values</t>
   </si>
   <si>
     <t>REG-MO-040</t>
@@ -787,8 +788,8 @@
 2. Toggle legend</t>
   </si>
   <si>
-    <t xml:space="preserve">Count-based graphs render
-Legend toggle restores</t>
+    <t xml:space="preserve">1. Count-based graphs render
+2. Legend toggle restores</t>
   </si>
   <si>
     <t>Hamburger options work independently on different device widgets</t>
@@ -803,11 +804,11 @@
 7. Confirm dashboard controls remain usable</t>
   </si>
   <si>
-    <t xml:space="preserve">Each device widget exposes its own hamburger menu
-Expected image export and chart interaction options are available
-Safe actions execute without corrupting other widgets
-Data-label/fullscreen state is restored
-No menu overlay blocks the dashboard</t>
+    <t xml:space="preserve">1. Each device widget exposes its own hamburger menu
+2. Expected image export and chart interaction options are available
+3. Safe actions execute without corrupting other widgets
+4. Data-label/fullscreen state is restored
+5. No menu overlay blocks the dashboard</t>
   </si>
   <si>
     <t>REG-MO-042</t>
@@ -821,8 +822,8 @@
 3. Cancel</t>
   </si>
   <si>
-    <t xml:space="preserve">Controls attached
-Cancel closes without applying</t>
+    <t xml:space="preserve">1. Controls attached
+2. Cancel closes without applying</t>
   </si>
   <si>
     <t>REG-MO-043</t>
@@ -836,9 +837,9 @@
 3. Clear/restore</t>
   </si>
   <si>
-    <t xml:space="preserve">Measurable refresh
-Original context restored
-Do not Save Filter</t>
+    <t xml:space="preserve">1. Measurable refresh
+2. Original context restored
+3. Do not Save Filter</t>
   </si>
   <si>
     <t>REG-MO-044</t>
@@ -852,8 +853,8 @@
 3. Restore</t>
   </si>
   <si>
-    <t xml:space="preserve">Filter applies
-Table reflects or empty state controlled</t>
+    <t xml:space="preserve">1. Filter applies
+2. Table reflects or empty state controlled</t>
   </si>
   <si>
     <t>REG-MO-045</t>
@@ -867,8 +868,8 @@
 3. Clear</t>
   </si>
   <si>
-    <t xml:space="preserve">Combination applies when options exist
-Context restored</t>
+    <t xml:space="preserve">1. Combination applies when options exist
+2. Context restored</t>
   </si>
   <si>
     <t>REG-MO-046</t>
@@ -881,7 +882,8 @@
 2. Observe Include/Exclude/Bots Only</t>
   </si>
   <si>
-    <t>Controls documented; no Save Filter</t>
+    <t xml:space="preserve">1. Controls documented
+2. no Save Filter</t>
   </si>
   <si>
     <t>Keyboard focus sample on primary controls</t>
@@ -890,7 +892,7 @@
     <t>1. Focus lookback, refresh, auto refresh, metric tab</t>
   </si>
   <si>
-    <t>Controls accept focus</t>
+    <t>1. Controls accept focus</t>
   </si>
   <si>
     <t>Responsive narrow desktop keeps essential controls reachable</t>
@@ -900,7 +902,7 @@
 2. Restore 1440</t>
   </si>
   <si>
-    <t>Lookback and Sitewide Totals remain reachable</t>
+    <t>1. Lookback and Sitewide Totals remain reachable</t>
   </si>
   <si>
     <t>Combination lookback + campaign metric + refresh without duplicates</t>
@@ -912,7 +914,7 @@
 4. Check duplicate hosts/cards</t>
   </si>
   <si>
-    <t>No duplicate graph hosts or campaignDiv IDs</t>
+    <t>1. No duplicate graph hosts or campaignDiv IDs</t>
   </si>
   <si>
     <t>Recover to original dashboard/lookback/metric context; page healthy</t>
@@ -922,8 +924,8 @@
 2. Confirm URL/title/widgets</t>
   </si>
   <si>
-    <t xml:space="preserve">Healthy Marketing Overview state
-Blocking errors annotated if any</t>
+    <t xml:space="preserve">1. Healthy Marketing Overview state
+2. Blocking errors annotated if any</t>
   </si>
   <si>
     <t>Blue Triangle Portal — Marketing Overview Regression Test Cases</t>
@@ -932,28 +934,22 @@
     <t>Profile / Site: US — GDC Test Site 2</t>
   </si>
   <si>
-    <t>Type: Regression. Do NOT Save Filter, create markers, edit/delete dashboards, or switch users. The controlled Hide Widget / Reset Widgets scenario must restore every hidden widget before continuing.</t>
-  </si>
-  <si>
-    <t>Do not hard-code dashboard name, lookback, campaign names, or metric totals.</t>
+    <t>Type: Regression (read-only). Prefer live UI; do not assert exact backend numeric values unless specified.</t>
   </si>
   <si>
     <t>Columns: Test Case ID | Type | Module | Submodule | Title | Steps | Expected Results | Status</t>
   </si>
   <si>
-    <t>Total cases: 50</t>
+    <t>Header style: bold white text on #1F4E79</t>
+  </si>
+  <si>
+    <t>Total cases: 50 (REG-MO-001 .. REG-MO-050)</t>
   </si>
   <si>
     <t>Automation: tests/regression_tests/US2/business-insights/improve-traffic/marketing-overview/marketing.overview.regression.spec.ts</t>
   </si>
   <si>
     <t>Execution status: Pass</t>
-  </si>
-  <si>
-    <t>Execution note: Latest automated run: 51 passed (50 REG-MO cases plus authentication). Source/Medium tables were unavailable. Soft findings: Orders tooltip retained currency, AOV occasionally remained on Revenue, and Sessions tooltip showed percentage formatting. See allure_reports/marketing-overview-report/index.html.</t>
-  </si>
-  <si>
-    <t>Live findings: Reset Widgets may restore positions without consistently unhiding every widget; use the hidden-widget panel for recovery. Source/Medium tables may be absent. Orders/Sessions tooltip units and AOV active-state behavior are recorded as soft findings when stale.</t>
   </si>
 </sst>
 </file>
@@ -970,7 +966,7 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="12"/>
     </font>
     <font>
       <b/>
@@ -989,7 +985,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2F5496"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
@@ -1018,15 +1014,17 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1369,427 +1367,424 @@
   <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="70" customWidth="1"/>
+    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="72" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2"/>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="E2"/>
-    </row>
-    <row r="3" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="2:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
+    <row r="4" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4" t="s">
+    <row r="5" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>6</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="4" t="s">
+    <row r="6" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>5</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="4" t="s">
+    <row r="7" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>4</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="4" t="s">
+    <row r="8" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="5">
         <v>3</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="4" t="s">
+    <row r="9" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="5">
         <v>3</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="4" t="s">
+    <row r="10" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="5">
         <v>3</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="4" t="s">
+    <row r="11" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="5">
         <v>3</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="4" t="s">
+    <row r="12" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="5">
         <v>2</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="4" t="s">
+    <row r="13" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="5">
         <v>2</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="4" t="s">
+    <row r="14" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="5">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="4" t="s">
+    <row r="15" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="5">
         <v>2</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="4" t="s">
+    <row r="16" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="5">
         <v>2</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C17" s="4" t="s">
+    <row r="17" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="5">
         <v>1</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C18" s="4" t="s">
+    <row r="18" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="5">
         <v>1</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C19" s="4" t="s">
+    <row r="19" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="5">
         <v>1</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C20" s="4" t="s">
+    <row r="20" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="5">
         <v>1</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21" s="4" t="s">
+    <row r="21" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="5">
         <v>1</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="5" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="4" t="s">
+    <row r="22" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="5">
         <v>1</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="4" t="s">
+    <row r="23" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="5">
         <v>1</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="4" t="s">
+    <row r="24" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="5">
         <v>1</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="5" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="4" t="s">
+    <row r="25" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="5">
         <v>1</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C26" s="4" t="s">
+    <row r="26" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="4">
+      <c r="D26" s="5">
         <v>1</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="4" t="s">
+    <row r="27" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="4">
+      <c r="D27" s="5">
         <v>1</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="28" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="4" t="s">
+    <row r="28" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D28" s="5">
         <v>1</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="2:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="4" t="s">
+    <row r="29" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D29" s="5">
         <v>1</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="5" t="s">
+    <row r="30" spans="2:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="6">
         <v>50</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" s="6" t="s">
         <v>60</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1801,1338 +1796,1339 @@
   <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="62" customWidth="1"/>
-    <col min="6" max="7" width="68" customWidth="1"/>
+    <col min="5" max="5" width="58" customWidth="1"/>
+    <col min="6" max="6" width="68" customWidth="1"/>
+    <col min="7" max="7" width="62" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+    <row r="2" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="B2" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="H2" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="H3" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="B4" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="5" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="H4" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="B5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="H5" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="B6" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="7" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="H6" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="B7" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="8" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="H7" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="B8" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="9" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="H8" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="B9" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="H9" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="B10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="H10" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="B11" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="H11" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="B12" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="H12" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="13" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="H12" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="B13" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="14" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="H13" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="B14" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="H14" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="H14" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="B15" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="16" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="H15" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="B16" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="H16" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="17" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="H16" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="B17" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="H17" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="18" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="H17" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="B18" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="19" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="H18" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="B19" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="H19" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="H19" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="B20" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="H20" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="21" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="H20" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" ht="124" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="B21" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="H21" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="22" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="H21" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="B22" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="H22" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="23" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="H22" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="B23" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H23" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="24" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="H23" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="B24" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="H24" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="H24" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="4" t="s">
+      <c r="B25" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="H25" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="26" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="H25" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="B26" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="H26" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="27" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+      <c r="H26" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="4" t="s">
+      <c r="B27" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="H27" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="28" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="H27" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" ht="140" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" s="4" t="s">
+      <c r="B28" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="H28" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="29" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="H28" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D29" s="4" t="s">
+      <c r="B29" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="G29" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="H29" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="30" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+      <c r="H29" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="B30" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="E30" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G30" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="H30" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="31" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="H30" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="B31" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="H31" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="32" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+      <c r="H31" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="4" t="s">
+      <c r="B32" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E32" s="4" t="s">
+      <c r="E32" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="G32" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="H32" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="33" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+      <c r="H32" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" ht="108" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33" s="4" t="s">
+      <c r="B33" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E33" s="4" t="s">
+      <c r="E33" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="G33" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="H33" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="34" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+      <c r="H33" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="4" t="s">
+      <c r="B34" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="E34" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="G34" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="H34" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="35" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+      <c r="H34" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" ht="108" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="4" t="s">
+      <c r="B35" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="E35" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F35" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="G35" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="H35" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="36" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
+      <c r="H35" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" ht="92" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="4" t="s">
+      <c r="B36" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="E36" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F36" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="G36" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="H36" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="37" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
+      <c r="H36" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" s="4" t="s">
+      <c r="B37" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G37" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="H37" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="38" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+      <c r="H37" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" ht="108" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="4" t="s">
+      <c r="B38" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="G38" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="H38" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="39" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="H38" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D39" s="4" t="s">
+      <c r="B39" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="E39" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="F39" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="G39" s="4" t="s">
+      <c r="G39" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="H39" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="40" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
+      <c r="H39" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40" s="4" t="s">
+      <c r="B40" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="F40" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="G40" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="H40" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="41" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
+      <c r="H40" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D41" s="4" t="s">
+      <c r="B41" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E41" s="4" t="s">
+      <c r="E41" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="F41" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="G41" s="5" t="s">
         <v>220</v>
       </c>
-      <c r="H41" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="42" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
+      <c r="H41" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="42" ht="124" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D42" s="4" t="s">
+      <c r="B42" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E42" s="4" t="s">
+      <c r="E42" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="F42" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="G42" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="H42" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="43" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
+      <c r="H42" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="43" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43" s="4" t="s">
+      <c r="B43" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E43" s="4" t="s">
+      <c r="E43" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="F43" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="G43" s="4" t="s">
+      <c r="G43" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="H43" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="44" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="4" t="s">
+      <c r="H43" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" s="4" t="s">
+      <c r="B44" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E44" s="4" t="s">
+      <c r="E44" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="F44" s="5" t="s">
         <v>230</v>
       </c>
-      <c r="G44" s="4" t="s">
+      <c r="G44" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="H44" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="45" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="4" t="s">
+      <c r="H44" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D45" s="4" t="s">
+      <c r="B45" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E45" s="4" t="s">
+      <c r="E45" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="F45" s="4" t="s">
+      <c r="F45" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="G45" s="4" t="s">
+      <c r="G45" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="H45" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="46" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="4" t="s">
+      <c r="H45" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D46" s="4" t="s">
+      <c r="B46" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E46" s="4" t="s">
+      <c r="E46" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="F46" s="4" t="s">
+      <c r="F46" s="5" t="s">
         <v>238</v>
       </c>
-      <c r="G46" s="4" t="s">
+      <c r="G46" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="H46" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="47" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="4" t="s">
+      <c r="H46" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="47" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47" s="4" t="s">
+      <c r="B47" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E47" s="4" t="s">
+      <c r="E47" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="F47" s="4" t="s">
+      <c r="F47" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="G47" s="4" t="s">
+      <c r="G47" s="5" t="s">
         <v>243</v>
       </c>
-      <c r="H47" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="48" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="4" t="s">
+      <c r="H47" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="48" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D48" s="4" t="s">
+      <c r="B48" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E48" s="4" t="s">
+      <c r="E48" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="F48" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="G48" s="4" t="s">
+      <c r="G48" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="H48" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="49" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
+      <c r="H48" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D49" s="4" t="s">
+      <c r="B49" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E49" s="4" t="s">
+      <c r="E49" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="F49" s="4" t="s">
+      <c r="F49" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="G49" s="4" t="s">
+      <c r="G49" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="H49" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="50" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
+      <c r="H49" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="50" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D50" s="4" t="s">
+      <c r="B50" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E50" s="4" t="s">
+      <c r="E50" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="F50" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="G50" s="4" t="s">
+      <c r="G50" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="H50" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="51" ht="100" customHeight="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
+      <c r="H50" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="51" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D51" s="4" t="s">
+      <c r="B51" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E51" s="4" t="s">
+      <c r="E51" s="5" t="s">
         <v>253</v>
       </c>
-      <c r="F51" s="4" t="s">
+      <c r="F51" s="5" t="s">
         <v>254</v>
       </c>
-      <c r="G51" s="4" t="s">
+      <c r="G51" s="5" t="s">
         <v>255</v>
       </c>
-      <c r="H51" s="4" t="s">
+      <c r="H51" s="5" t="s">
         <v>72</v>
       </c>
     </row>
@@ -3152,14 +3148,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>256</v>
       </c>
     </row>
@@ -3190,27 +3186,12 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
         <v>263</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>